<commit_message>
Add Bolts tab with fastener reference data
- Bolt/anchor rod grades (A307, A325, A490, F1554 Gr36/55/105)
- Standard hole sizes (STD/OVS/SSLOT/LSLOT) per AISC Table J3.3
- Min edge distance and bolt spacing per AISC Table J3.4
- Approximate snug-tight torque values for A325/A490

https://claude.ai/code/session_01WHBFwynTiNtj9dpYbYeF6i
</commit_message>
<xml_diff>
--- a/steel_detailing_reference.xlsx
+++ b/steel_detailing_reference.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Handrail" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Pipe Supports" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Platforms" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Bolts" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7368,4 +7369,1102 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C00000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BOLT &amp; ANCHOR ROD GRADES  (AISC / ASTM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Spec</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Fy (ksi)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Fu (ksi)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Shear (ksi)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Tension (ksi)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>A307</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Low carbon</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>27.0</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Non-structural; anchor bolts, light connections</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>A325</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Med carbon</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>90.0</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Standard structural bolt; most common</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>A490</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Alloy steel</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>67.5</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>112.5</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>High-strength; heavier connections</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>F1554 Gr36</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Low carbon</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Anchor rods; weldable</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>F1554 Gr55</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Med carbon</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Anchor rods; higher strength</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>F1554 Gr105</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Alloy</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Anchor rods; heavy equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>A36 Threaded</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Low carbon</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>All-thread rod; misc bracing/hangers</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>STANDARD HOLE SIZES  (AISC Table J3.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Bolt Dia</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>STD Hole</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>OVS Hole</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>SSLOT Width</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>SSLOT Length</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>LSLOT Width</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>LSLOT Length</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>1/2"</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>9/16"</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>5/8"</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>9/16"</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>11/16"</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>9/16"</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>1-1/4"</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>5/8"</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>11/16"</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>13/16"</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>11/16"</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>7/8"</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>11/16"</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>1-9/16"</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>3/4"</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>13/16"</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>15/16"</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>13/16"</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>1"</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>13/16"</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>1-7/8"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>7/8"</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>15/16"</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>1-1/16"</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>15/16"</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>1-1/8"</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>15/16"</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>2-3/16"</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1"</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>1-1/16"</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>1-1/4"</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>1-1/16"</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>1-5/16"</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>1-1/16"</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>2-1/2"</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>1-1/8"</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>1-3/16"</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>1-3/8"</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>1-3/16"</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>1-7/16"</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>1-3/16"</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>2-13/16"</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>1-1/4"</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>1-5/16"</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>1-1/2"</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>1-5/16"</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>1-9/16"</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>1-5/16"</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>3-1/8"</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>MIN EDGE DISTANCE &amp; BOLT SPACING  (AISC Table J3.4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Bolt Dia</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Min Edge (sheared)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Min Edge (rolled/saw)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Min Spacing (3x dia)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>1/2"</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>7/8"</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>3/4"</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>1-1/2"</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>5/8"</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>1-1/8"</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>7/8"</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>1-7/8"</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>3/4"</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>1-1/4"</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>1"</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>2-1/4"</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>7/8"</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>1-1/2"</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>1-1/8"</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>2-5/8"</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr"/>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>1"</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>1-3/4"</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>1-1/4"</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>3"</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+      <c r="G27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>1-1/8"</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>2"</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>1-1/2"</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>3-3/8"</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr"/>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>1-1/4"</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>2-1/4"</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>1-5/8"</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>3-3/4"</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>APPROXIMATE SNUG-TIGHT TORQUE  (Reference only — follow approved ITP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Bolt Dia</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Grip Range</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>A325 Torque (ft-lbs)</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>A490 Torque (ft-lbs)</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>1/2"</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr"/>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>3/16" – 1"</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>107</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>5/8"</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr"/>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>3/16" – 1"</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>3/4"</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>1/4" – 1-1/2"</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>375</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>7/8"</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr"/>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>1/4" – 2"</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>490</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>612</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>1"</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr"/>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>1/4" – 2"</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>730</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>912</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>1-1/8"</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr"/>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>3/8" – 2"</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>1312</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>1-1/4"</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr"/>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>3/8" – 2"</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>1460</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>1825</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr"/>
+      <c r="G39" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>• STD = Standard hole | OVS = Oversized | SSLOT = Short-slot | LSLOT = Long-slot</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>• A325 and A490 are now superseded by ASTM F3125 Gr A325/A490 — same dimensions/strengths</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>• Min spacing = 2-2/3 × bolt dia (preferred 3×); min edge = per table above</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>• For slip-critical connections use Class A or B faying surface — see engineer</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>• Torque values are approximate — always follow the project Inspection &amp; Test Plan (ITP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>• F1554 anchor rods: embed length = 12× dia minimum unless engineer specifies otherwise</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A42:G42"/>
+    <mergeCell ref="A46:G46"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Welds, Converter, and References tabs with clickable links
- Welds tab: AWS D1.1 min fillet sizes, max single-pass, edge limits,
  prequalified joint details, electrode-base metal match table
- Converter tab: live calculators for length/weight/pressure/stress/temp
  plus static conversion factor reference table
- References tab: all 18 standards cited in workbook with clickable
  hyperlinks to source (OSHA/AISC free; ASME/AWS/ASTM purchase pages)

11 tabs total. References tab lets Steven show exactly where every
number came from when questioned on site or in the shop.

https://claude.ai/code/session_01WHBFwynTiNtj9dpYbYeF6i
</commit_message>
<xml_diff>
--- a/steel_detailing_reference.xlsx
+++ b/steel_detailing_reference.xlsx
@@ -15,6 +15,9 @@
     <sheet name="Pipe Supports" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Platforms" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Bolts" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Welds" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Converter" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="References" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,12 +26,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,6 +77,13 @@
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -164,10 +175,11 @@
       </bottom>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -212,9 +224,23 @@
     <xf numFmtId="166" fontId="6" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="167" fontId="6" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -2778,6 +2804,1227 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0000B0F0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>UNIT CONVERTER  (Enter values in YELLOW cells — results auto-calculate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>LENGTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Inches:</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>→  Feet:</t>
+        </is>
+      </c>
+      <c r="D3" s="11">
+        <f>B3/12</f>
+        <v/>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>→  mm:</t>
+        </is>
+      </c>
+      <c r="F3" s="11">
+        <f>B3*25.4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>→  Meters:</t>
+        </is>
+      </c>
+      <c r="D4" s="17">
+        <f>B3*0.0254</f>
+        <v/>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>→  cm:</t>
+        </is>
+      </c>
+      <c r="F4" s="11">
+        <f>B3*2.54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>WEIGHT / FORCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Pounds (lbs):</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>→  Kilograms:</t>
+        </is>
+      </c>
+      <c r="D7" s="11">
+        <f>B7*0.453592</f>
+        <v/>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>→  kips:</t>
+        </is>
+      </c>
+      <c r="F7" s="11">
+        <f>B7/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>→  kN:</t>
+        </is>
+      </c>
+      <c r="D8" s="11">
+        <f>B7*0.004448</f>
+        <v/>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>→  Newtons:</t>
+        </is>
+      </c>
+      <c r="F8" s="13">
+        <f>B7*4.44822</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>LOAD / PRESSURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>lb/sq ft (psf):</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>→  kPa:</t>
+        </is>
+      </c>
+      <c r="D11" s="11">
+        <f>B11*0.047880</f>
+        <v/>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>→  psi:</t>
+        </is>
+      </c>
+      <c r="F11" s="11">
+        <f>B11/144</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>→  ksf:</t>
+        </is>
+      </c>
+      <c r="D12" s="17">
+        <f>B11/1000</f>
+        <v/>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>→  Pa:</t>
+        </is>
+      </c>
+      <c r="F12" s="13">
+        <f>B11*47.880</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>STRESS (ksi ↔ MPa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>ksi (kips/in²):</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>→  MPa:</t>
+        </is>
+      </c>
+      <c r="D15" s="18">
+        <f>B15*6.89476</f>
+        <v/>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>→  psi:</t>
+        </is>
+      </c>
+      <c r="F15" s="12">
+        <f>B15*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>TEMPERATURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>°F:</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>→  °C:</t>
+        </is>
+      </c>
+      <c r="D18" s="13">
+        <f>(B18-32)*5/9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>COMMON CONVERSION FACTORS (Quick Reference)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Multiply by</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>1 inch</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>millimeters</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>25.4</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>1 foot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>millimeters</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>304.8</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="5" t="inlineStr"/>
+      <c r="F23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>1 foot</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>meters</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>0.3048</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>1 lb</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>kilograms</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>0.4536</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr"/>
+      <c r="E25" s="5" t="inlineStr"/>
+      <c r="F25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>1 kip</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>kilonewtons</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>4.4482</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>1 psf</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>kPa</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>0.04788</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="5" t="inlineStr"/>
+      <c r="F27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>1 ksi</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>6.8948</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>1 lb/ft</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>kg/m</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>1.4882</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr"/>
+      <c r="E29" s="5" t="inlineStr"/>
+      <c r="F29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>1 in²</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>mm²</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>645.16</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>1 in³</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>mm³</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>16387.1</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr"/>
+      <c r="E31" s="5" t="inlineStr"/>
+      <c r="F31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>1 in⁴</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>mm⁴</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>416231.0</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A20:F20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00404040"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STANDARDS &amp; CODE REFERENCES  — Where the data in this workbook comes from</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Full Title</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Used In Tab</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>What It Covers</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Access</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Click to Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>AISC SCM 16th Ed</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Steel Construction Manual, 16th Edition</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Part 1 — Section Tables</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>W/C/Angle/HSS/Pipe properties; connection design</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Free (login req.)</t>
+        </is>
+      </c>
+      <c r="F3" s="19" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>AISC Table J3.3</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>SCM Table J3.3 — Bolt Hole Sizes</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Bolts tab</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>STD, OVS, SSLOT, LSLOT hole dimensions for all bolt diameters</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Free (login req.)</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>AISC Table J3.4</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>SCM Table J3.4 — Minimum Edge Distances</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Bolts tab</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Min edge distance from bolt center to edge of connected part</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Free (login req.)</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>AWS D1.1</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Structural Welding Code — Steel</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Welds tab</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Prequalified joints, fillet weld sizes, electrode matching, preheat</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ASME B36.10M</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Welded and Seamless Wrought Steel Pipe</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Pipe tab</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Pipe OD, wall thickness, ID, weight for all NPS sizes and schedules</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>OSHA 1910.29</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Fall Protection Systems — Walking-Working Surfaces</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Handrail tab</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>42" top rail, 21" mid rail, 200 lb strength, toeboard requirements</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>OSHA 1926.502</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Fall Protection Systems — Construction</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Handrail tab</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Construction site fall protection; same rail heights as 1910.29</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>FREE</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>ASCE 7-22</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Minimum Design Loads and Associated Criteria</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Platforms tab</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Live loads: 50 psf industrial platform, 40 psf maintenance only</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ASTM A36</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Standard Spec for Carbon Structural Steel</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Materials tab</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Fy=36 ksi, Fu=58-80 ksi; plates, shapes, bars</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>ASTM A572</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>HSLA Structural Steel (Gr 42/50/55/60/65)</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Materials tab</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Gr50: Fy=50, Fu=65; W-shapes, beams, columns</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>ASTM A992</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Structural Steel Shapes — W-Shapes</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Materials tab</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Fy=50 min, Fu=65; Fy/Fu &lt;= 0.85; current standard for W-shapes</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>ASTM A500</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Cold-Formed Welded/Seamless Structural Tubing</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Materials tab</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Gr B: Fy=46, Fu=58; Gr C: Fy=50, Fu=62; square/rect HSS</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>ASTM A53</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Pipe, Steel, Black and Hot-Dipped</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Pipe &amp; Materials tabs</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Gr B: Fy=35, Fu=60; ERW or seamless; structural pipe</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>ASTM A106</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Seamless Carbon Steel Pipe for High-Temp Service</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Pipe &amp; Materials tabs</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Gr B: Fy=35, Fu=60; seamless only; process/pressure piping</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>ASTM F3125 (A325/A490)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>High Strength Structural Bolts (supersedes A325/A490)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Bolts tab</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Gr A325: Fy=92, Fu=120; Gr A490: Fy=130, Fu=150</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>ASTM F1554</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Anchor Bolts, Steel, 36/55/105 ksi Yield</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Bolts tab</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Anchor rods for base plates; Gr36 is weldable</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>ASTM A307</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Carbon Steel Bolts, Studs — 60 ksi</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Bolts tab</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Low-strength; non-structural connections, anchor bolts</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>MSS SP-58</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Pipe Hangers and Supports — Materials/Design</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Pipe Supports tab</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Types 1-42 pipe clamp/support configurations</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Purchase required</t>
+        </is>
+      </c>
+      <c r="F20" s="20" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>• FREE = Available at no cost online (click link to open directly)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>• Purchase required = Paid standard; link goes to purchase/info page</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>• AISC Steel Construction Manual is FREE to download with a free account at aisc.org — highly recommended</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>• OSHA standards (1910 and 1926) are always free at osha.gov — bookmark these</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>• AWS D1.1 and ASME B36.10 require purchase — your company may have copies in the office</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>• When someone asks 'where did you get that number?' — point them to this tab and the linked source</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A25:F25"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId18"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -8467,4 +9714,749 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF6600"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>WELD REFERENCE — AWS D1.1 Structural Welding Code (Steel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MIN FILLET WELD SIZE (AWS D1.1 Table 8.8)  — based on THICKER part joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Base Metal Thickness (thicker part)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Min Fillet Weld Size</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>To 1/4" incl.</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>1/8"</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Do not weld thinner than 1/8"</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Over 1/4" to 1/2"</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>3/16"</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Most common shop minimum</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Over 1/2" to 3/4"</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>1/4"</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Over 3/4"</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>5/16"</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Minimum for heavy plate</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>MAX SINGLE-PASS FILLET WELD SIZE (AWS D1.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Max Single-Pass Size</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Flat / Horizontal</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>5/16"</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>AWS D1.1 limit per pass</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Vertical</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>1/4"</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr"/>
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Overhead</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>1/4"</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>MAX FILLET WELD SIZE ALONG EDGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Edge Thickness</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Max Weld Size</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>&lt; 1/4" thick edge</t>
+        </is>
+      </c>
+      <c r="B17" s="4">
+        <f> plate thickness</f>
+        <v/>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Full-thickness weld allowed</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>&gt;= 1/4" thick edge</t>
+        </is>
+      </c>
+      <c r="B18" s="6">
+        <f> plate thickness - 1/16"</f>
+        <v/>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Must leave 1/16" land</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>PREQUALIFIED JOINT DETAILS (AWS D1.1) — Reference Only</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Joint Type</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>AWS Symbol</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Root Opening</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Groove Angle</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Square Groove, no gap</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>B-L1a</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>t &lt;= 5/16" SMAW; &lt;= 3/8" SAW</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Square Groove, w/ gap</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>B-L1b</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>1/4" max</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Both sides or back-gouge</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Single-V, 60°</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>B-U1a</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>0–1/4"</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>60°</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Most common groove weld</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr"/>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Single-Bevel, 45°</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>B-U2</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>0–1/8"</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>45°</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>One-sided access joints</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr"/>
+      <c r="G25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Single-V, 45°</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>B-U1</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>0–1/8"</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>45°</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Double-V, 60°</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>B-U1b</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>0–1/8"</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>60°</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Both sides; balanced distortion</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr"/>
+      <c r="G27" s="5" t="inlineStr"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>ELECTRODE — BASE METAL MATCH TABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Base Metal</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Min Fu (ksi)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Recommended Electrode</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>A36</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>E70xx</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Overmatch is fine and common</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+      <c r="G31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>A572 Gr50</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>E70xx</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>70 ksi filler satisfies 65 ksi base</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr"/>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>A992</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>E70xx</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Same as A572 Gr50 in practice</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>A500 B/C</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>E70xx</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>E7018 preferred for thicker walls</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>A53-B</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>E70xx</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>E7018 (low hydrogen) per most WPS</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>A106-B</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>E7018</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Preheat per AWS D1.1 when t &gt; 1"</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>• Fillet weld size on drawing = LEG size (not throat). Throat = 0.707 × leg for equal-leg fillet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>• Always use the THICKER part to determine minimum weld size — not the thinner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>• E7018 is low-hydrogen; keep electrodes in oven or rod oven — discard if exposed &gt; 4 hrs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>• Preheat required per AWS D1.1 Table 3.2 when CEQ &gt; 0.40 or plate t &gt; 1.5" A36.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>• WPS = Welding Procedure Specification — always weld to an approved WPS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>• PQR = Procedure Qualification Record — proves the WPS works.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>• AWS D1.1 is the governing code for structural steel welding in most fabrication shops.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A42:G42"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>